<commit_message>
Add bootstrap CIs and fix effect size to rank-biserial r
- Replace ad-hoc median/SD effect size with matched-pairs rank-biserial
  correlation (Rosenthal 1991), the standard measure for Wilcoxon tests
- Add 10k-resample bootstrap 95% CIs on median time difference and
  Jackson/Dalton split percentage
- Document both additions in README statistical tests section

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBCJ_Analysis_Results.xlsx
+++ b/FBCJ_Analysis_Results.xlsx
@@ -3034,80 +3034,80 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Orock, Kendall, Orock, Matt and Jenn, Orock, Samantha</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>2739 Mason Street, SW</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Massillon</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>44646</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F33" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G33" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I33" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="2" t="n">
+      <c r="G33" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="4" t="n">
         <v>10.8</v>
       </c>
-      <c r="K33" s="2" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="L33" s="2" t="n">
+      <c r="K33" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="L33" s="4" t="n">
         <v>13.3</v>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="M33" s="4" t="n">
         <v>14.8</v>
       </c>
-      <c r="N33" s="2" t="n">
+      <c r="N33" s="4" t="n">
         <v>-2.5</v>
       </c>
-      <c r="O33" s="2" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="P33" s="3" t="n">
-        <v>0.268</v>
-      </c>
-      <c r="Q33" s="3" t="n">
-        <v>0.732</v>
-      </c>
-      <c r="R33" s="2" t="inlineStr">
+      <c r="O33" s="4" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="P33" s="5" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="Q33" s="5" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="R33" s="4" t="inlineStr">
         <is>
           <t>Dalton</t>
         </is>
       </c>
-      <c r="S33" s="2" t="inlineStr">
+      <c r="S33" s="4" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="T33" s="2" t="inlineStr">
-        <is>
-          <t>Low (Straight-line est.)</t>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -22046,7 +22046,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>261</t>
         </is>
       </c>
     </row>
@@ -22058,7 +22058,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
     </row>
@@ -22130,7 +22130,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>173 (66.5%)</t>
+          <t>173 (66.3%)</t>
         </is>
       </c>
     </row>
@@ -22142,7 +22142,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>37 (14.2%)</t>
+          <t>38 (14.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>